<commit_message>
[看板] 02/03 部署主线 voxslice + 验收
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-17.xlsx
+++ b/docs/progress/显性目的进度_2026-10-17.xlsx
@@ -8522,7 +8522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J176"/>
+  <dimension ref="A1:J180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9817,101 +9817,101 @@
     </row>
     <row r="57">
       <c r="A57" s="17" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>回归</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>全套</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>上板故障演练 14/14 PASS (povnetd 1.2): 装后重启 88 s; 杀 sshd/mdns/povnetd 60/7/72 s; 杀 wpa ×3 12/32/22 s; 关网卡 ×3 22/32/34 s; 错 SSID→热点→自回 545 s; 看门狗复位 2 项 60/220 s 找回且记非正常结束。用户要求 '不插串口永远连得上' 达成; 合主线回归中</t>
+          <t>最新主线 fdb63f4 全套 19 套: 15 过; v2_map G4 / v2_bridge S 为守护误报 (D27b 时序摘要) 已修 d4a4e3a; 🔴 d19 O4_fake / d20_smooth S2 真回归: 假转本地播放换网格率 = 1×转速 (半圈换未生效), 10-16 3cb39fc 时 d19 PASS → 疑 D20e --pl-gate, 已退回 D20e agent 查修</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22c.board.log</t>
+          <t>dr1v90 ~/full_*.log</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="17" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B58" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46312</v>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>修复</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D20e</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>不插串口永远连得上 合主线 (上板演练 14/14; 合并回归 D22/rotor_ops/D18/D13/live_push 全过, D13 补丁比较口径剔除 D22 块)。串口可永久拔</t>
+          <t>本地播放半圈换回归修复合主线 86caee5 (复验 d19 16/0, d20_smooth, d20d, d20e V1-V5 全过): 根因 2cd422a 对齐放行 (--pl-gate) 对本地帧也生效, 本地 15 fps+margin 0.9 时 m=2 压成 1×转速; 改为只作用推流帧; 02 开机演示配置 (10 fps/20/1.0) 推算不受影响; voxslice 新 md5 63e7afea, 下次部署换</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 slice/SPEC.md §13.2</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="17" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>长跑</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>上板 PASS: 假转 5→20→5 斜坡换档 2 次 + 强制轮换 6 次, 跨圈写 0, 超时 0, 对拍 2/0 与 12/0, 完成率 100%, 收尾回默认 0x20471019 (测试解析同 D19 修正)。合并分支 task/merge-d21 全回归 12 套进行中</t>
+          <t>02 24 h 产品配置长跑 PASS 10/10 (主线 8eced5a, PLV=0 max-fps 20 margin 1.0): 停摆 0/死 0, 10 s 窗口完成率最低 100%, 最差小时未完成 0.0011%, 推流 29 段 rc 0 均 16.8 帧/s, 停推 32 次全 300 s 回本地, RSS 23.1→23.1 MB; 注: PC 侧 D 盘 EIO 致 soak.sh 末段退出 (板上照常跑满并自恢复, 日志手动取回判读), ping 只记前 46 次, push.txt 少 3 段</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d21.board5.log</t>
+          <t>progress/soak_v0/1016_wkend_24h</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="17" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B60" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46312</v>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>部署</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>每圈片数随转速换档合主线 (全回归 12 套通过; D18 V3 允许卡上默认 kit=D19 落后仓库 RTL=D21); 主线 voxslice 已修 sub01 隐患。下一步: V1 12-bit 位流按主线 (D19+D21+D8) 重综合</t>
+          <t>02/03 卡上 voxslice 换主线 86caee5 版 (63e7afea, 旧版留 .bak-0717), 重启验收: 03 6/6 PASS; 02 A5 首次 1243 帧/90 s (&lt;1260, 开机后 20 s 内推流) 其余全过, 随后连推 3 次 1351/1351/1349 帧 = 满 15 帧/s → 判为开机初期偶发</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>progress/v0_accept/accept_1017_*.log</t>
         </is>
       </c>
     </row>
@@ -9919,24 +9919,24 @@
       <c r="A61" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B61" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>内容帧率跟转速 voxlive --fps auto 合主线 d3f16f3 (默认不变; 主机空闲时离线复验 PASS, 之前失败为主机忙)。上板 A/B (583 rpm 固定 15 vs auto+板 20/1.0) 进行中</t>
+          <t>上板故障演练 14/14 PASS (povnetd 1.2): 装后重启 88 s; 杀 sshd/mdns/povnetd 60/7/72 s; 杀 wpa ×3 12/32/22 s; 关网卡 ×3 22/32/34 s; 错 SSID→热点→自回 545 s; 看门狗复位 2 项 60/220 s 找回且记非正常结束。用户要求 '不插串口永远连得上' 达成; 合主线回归中</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>~/rv_d22c.board.log</t>
         </is>
       </c>
     </row>
@@ -9944,24 +9944,24 @@
       <c r="A62" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B62" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B62" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>上板 A/B (假转 583 rpm, 无对拍, 逐帧): A 默认 (推 15 + 板 15/0.9) 14.85/s, 间隔 p50/p95 51.5/103 ms, 节拍偏差 p50/p95 23%/55%; B (推 auto + 板 max-fps 20 / margin 1.0) 19.14/s, 间隔 51.4/51.8 ms, 偏差 0%/1%, 最长 206 ms。B 明显更流畅; 测 C (转速取自板遥测) 后决定改开机默认</t>
+          <t>不插串口永远连得上 合主线 (上板演练 14/14; 合并回归 D22/rotor_ops/D18/D13/live_push 全过, D13 补丁比较口径剔除 D22 块)。串口可永久拔</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_A fps_B</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -9969,24 +9969,24 @@
       <c r="A63" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B63" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>测 C: 不手填转速时 auto 拿不到转速 → 退回 15 fps (povstat UDP 在 WSL NAT 收不到; 且 V0 2047 PL 位流遥测本无转速)。开 D20d: 推流 TCP ACK 扩展回传转速 (新旧兼容) + 默认改 板 max-fps 20/margin 1.0、推流 auto; 同时开 D10 V1 12-bit 位流按主线重综合</t>
+          <t>上板 PASS: 假转 5→20→5 斜坡换档 2 次 + 强制轮换 6 次, 跨圈写 0, 超时 0, 对拍 2/0 与 12/0, 完成率 100%, 收尾回默认 0x20471019 (测试解析同 D19 修正)。合并分支 task/merge-d21 全回归 12 套进行中</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_C</t>
+          <t>~/rv_d21.board5.log</t>
         </is>
       </c>
     </row>
@@ -9994,24 +9994,24 @@
       <c r="A64" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B64" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B64" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>D20d</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>推流 ACK 扩展回传转速 (帧头 flags bit15 请求 → 板回 0x07+rps×100+max-fps+margin+半圈标志; 新旧三种组合逐字节兼容) + 默认 板 max-fps 20/margin 1.0、推流 --fps auto (不用手填): 离线假转 583 rpm 自动锁 19.49/s std 0.2 ms。复验 + 上板 D 组进行中</t>
+          <t>每圈片数随转速换档合主线 (全回归 12 套通过; D18 V3 允许卡上默认 kit=D19 落后仓库 RTL=D21); 主线 voxslice 已修 sub01 隐患。下一步: V1 12-bit 位流按主线 (D19+D21+D8) 重综合</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20d-ackrps db4ec93</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10019,24 +10019,24 @@
       <c r="A65" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B65" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B65" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>V1 主控 12-bit 位流按主线重综合 8 档时序全收住 (回板主用 ul800_p1_b12 md5 023e6582, 替换作废 df4f0bea); 修 D8 引入的 build.sh set -e 静默退出; 2 期 MAXMISS 系命令配错 (12-bit@800M 本就超片周期), 非回归; 回板步骤 BOARD_DAY.md。注: V1 线速 800M (派活单写 1.2G 是主会话笔误); 缺口: V1 真内容板端通路 (voxslice 只支持 2047 后端) 待立项</t>
+          <t>内容帧率跟转速 voxlive --fps auto 合主线 d3f16f3 (默认不变; 主机空闲时离线复验 PASS, 之前失败为主机忙)。上板 A/B (583 rpm 固定 15 vs auto+板 20/1.0) 进行中</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d10-v1bit 9a9acf8</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10046,22 +10046,22 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>测量</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>D20d</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>上板 D 组 (不手填任何参数): 推流经 ACK 扩展自动拿到转速并锁 19.4 帧/s ✅; 但间隔 p95 103 ms (&gt;5% 帧翻倍), 不如手填转速的 B 组 (p95 51.8) —— 估计转速与实际微差导致周期性滑格, 需相位锁定 (跟板端 ACK 节奏) 作后续。离线复验 (指定 BASE) PASS, 合主线回归中</t>
+          <t>上板 A/B (假转 583 rpm, 无对拍, 逐帧): A 默认 (推 15 + 板 15/0.9) 14.85/s, 间隔 p50/p95 51.5/103 ms, 节拍偏差 p50/p95 23%/55%; B (推 auto + 板 max-fps 20 / margin 1.0) 19.14/s, 间隔 51.4/51.8 ms, 偏差 0%/1%, 最长 206 ms。B 明显更流畅; 测 C (转速取自板遥测) 后决定改开机默认</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_D</t>
+          <t>soak_runs/fps_A fps_B</t>
         </is>
       </c>
     </row>
@@ -10069,24 +10069,24 @@
       <c r="A67" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B67" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B67" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>D20d</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>ACK 回传转速 + 默认推流 auto / 板 20/1.0 合主线 (合并回归 7 套通过)。卡上部署尚未更新 (下次装卡带上); 后续: 相位锁定消 5% 滑格</t>
+          <t>测 C: 不手填转速时 auto 拿不到转速 → 退回 15 fps (povstat UDP 在 WSL NAT 收不到; 且 V0 2047 PL 位流遥测本无转速)。开 D20d: 推流 TCP ACK 扩展回传转速 (新旧兼容) + 默认改 板 max-fps 20/margin 1.0、推流 auto; 同时开 D10 V1 12-bit 位流按主线重综合</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>soak_runs/fps_C</t>
         </is>
       </c>
     </row>
@@ -10096,22 +10096,22 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>部署</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D20d</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>卡上部署更新到主线 1d23e50 (voxslice md5 ecdc246f = 主线, show_boot max-fps 20 / margin 1.0, QoS 0x0F, PL 0x20471019, D22 povreach); D19 上板假转扫点 PASS</t>
+          <t>推流 ACK 扩展回传转速 (帧头 flags bit15 请求 → 板回 0x07+rps×100+max-fps+margin+半圈标志; 新旧三种组合逐字节兼容) + 默认 板 max-fps 20/margin 1.0、推流 --fps auto (不用手填): 离线假转 583 rpm 自动锁 19.49/s std 0.2 ms。复验 + 上板 D 组进行中</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>~/rv_deploy.board.log</t>
+          <t>dr1v90 task/d20d-ackrps db4ec93</t>
         </is>
       </c>
     </row>
@@ -10119,9 +10119,9 @@
       <c r="A69" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B69" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
@@ -10131,12 +10131,12 @@
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>V1 主控位流按主线重综合合主线 (复验 5/5: 构建记录/联合仿真/上行回归/MAXMISS 说明); 回板步骤 d10_v1bit/BOARD_DAY.md</t>
+          <t>V1 主控 12-bit 位流按主线重综合 8 档时序全收住 (回板主用 ul800_p1_b12 md5 023e6582, 替换作废 df4f0bea); 修 D8 引入的 build.sh set -e 静默退出; 2 期 MAXMISS 系命令配错 (12-bit@800M 本就超片周期), 非回归; 回板步骤 BOARD_DAY.md。注: V1 线速 800M (派活单写 1.2G 是主会话笔误); 缺口: V1 真内容板端通路 (voxslice 只支持 2047 后端) 待立项</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 task/d10-v1bit 9a9acf8</t>
         </is>
       </c>
     </row>
@@ -10146,22 +10146,22 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>验收</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D20d</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>用户重启板子后 V0 验收 6/6 PASS (不插串口): 按名字找回 / 守护进程齐 (voxslice povnetd povreach povmdns povstat) / 开机默认 PL+QoS 0x0F+位流 0x20471019 / WiFi -55 dBm ping 30 丢 0 / 推流 90 s 1339 帧=14.9 帧/s 对端关闭 / 推后 voxslice 不变。首跑遇 D 盘 EIO 中断后重跑; A5 判读正则修正</t>
+          <t>上板 D 组 (不手填任何参数): 推流经 ACK 扩展自动拿到转速并锁 19.4 帧/s ✅; 但间隔 p95 103 ms (&gt;5% 帧翻倍), 不如手填转速的 B 组 (p95 51.8) —— 估计转速与实际微差导致周期性滑格, 需相位锁定 (跟板端 ACK 节奏) 作后续。离线复验 (指定 BASE) PASS, 合主线回归中</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/</t>
+          <t>soak_runs/fps_D</t>
         </is>
       </c>
     </row>
@@ -10169,24 +10169,24 @@
       <c r="A71" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B71" s="6" t="inlineStr">
-        <is>
-          <t>开工</t>
+      <c r="B71" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>D20e/D23</t>
+          <t>D20d</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>D20e 推流相位锁定 (消 auto 模式 5% 滑格) + D23 V1 真内容板端通路 并行开工; 用户新提: 开机默认动画要有立方体动图 (待做)</t>
+          <t>ACK 回传转速 + 默认推流 auto / 板 20/1.0 合主线 (合并回归 7 套通过)。卡上部署尚未更新 (下次装卡带上); 后续: 相位锁定消 5% 滑格</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20e-phaselock task/d23-v1content</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10194,24 +10194,24 @@
       <c r="A72" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B72" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>部署</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>D24</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>用户: 开机动画就用现在这个 (geo_loop, 含线框立方体), 不换; D26 V2 位流构建放行, 主会话后台跑; 新板定名 DR1M90-03, 拷卡包 card_kit_dr1m90-03 待用户管理员运行 make_card.ps1</t>
+          <t>卡上部署更新到主线 1d23e50 (voxslice md5 ecdc246f = 主线, show_boot max-fps 20 / margin 1.0, QoS 0x0F, PL 0x20471019, D22 povreach); D19 上板假转扫点 PASS</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>用户</t>
+          <t>~/rv_deploy.board.log</t>
         </is>
       </c>
     </row>
@@ -10226,12 +10226,12 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>D23</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>V1 显示后端 voxslice --disp 2260 合主线 a41d63b (独立复验 24/0, 合并后回归 d21/d23 过)</t>
+          <t>V1 主控位流按主线重综合合主线 (复验 5/5: 构建记录/联合仿真/上行回归/MAXMISS 说明); 回板步骤 d10_v1bit/BOARD_DAY.md</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
@@ -10244,24 +10244,24 @@
       <c r="A74" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B74" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>验收</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>D20e</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>推流相位锁定合主线 c80f5fb: 583 rpm 滑格 5.2%→0.19%, 900 rpm 22%→0.12% (p95 = 理想间隔); 代价 延迟 120→170-250 ms (--phaselock off 可回老行为)</t>
+          <t>用户重启板子后 V0 验收 6/6 PASS (不插串口): 按名字找回 / 守护进程齐 (voxslice povnetd povreach povmdns povstat) / 开机默认 PL+QoS 0x0F+位流 0x20471019 / WiFi -55 dBm ping 30 丢 0 / 推流 90 s 1339 帧=14.9 帧/s 对端关闭 / 推后 voxslice 不变。首跑遇 D 盘 EIO 中断后重跑; A5 判读正则修正</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>progress/v0_accept/</t>
         </is>
       </c>
     </row>
@@ -10271,22 +10271,22 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>部署</t>
+          <t>开工</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D20e/D23</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>02 卡上 voxslice 换 D20e 版 (ba243d71, 旧版留 .bak-d20e), 重启后 V0 验收 6/6 PASS (推流 1326 帧/90 s, WiFi -44 dBm 丢 0)</t>
+          <t>D20e 推流相位锁定 (消 auto 模式 5% 滑格) + D23 V1 真内容板端通路 并行开工; 用户新提: 开机默认动画要有立方体动图 (待做)</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/accept_1016_d20e.log</t>
+          <t>dr1v90 task/d20e-phaselock task/d23-v1content</t>
         </is>
       </c>
     </row>
@@ -10294,24 +10294,24 @@
       <c r="A76" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B76" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B76" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>KR7.3/D24</t>
+          <t>D24</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>KR7.3 16 位计数回绕修正合主线 (存档无原始计数, 99.84% 无法重算; 38/57 转动行待核); D24 立方体候选合主线, 用户定开机保持 geo_loop</t>
+          <t>用户: 开机动画就用现在这个 (geo_loop, 含线框立方体), 不换; D26 V2 位流构建放行, 主会话后台跑; 新板定名 DR1M90-03, 拷卡包 card_kit_dr1m90-03 待用户管理员运行 make_card.ps1</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>用户</t>
         </is>
       </c>
     </row>
@@ -10319,24 +10319,24 @@
       <c r="A77" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B77" s="6" t="inlineStr">
-        <is>
-          <t>硬件</t>
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>D23</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>第二块板: 公司 DLP 拦 TF 卡文件写入 → WSL 做 512 MB 镜像 + host/flash_card_raw.ps1 块级写, 读回 PASS; 等上电按名字找</t>
+          <t>V1 显示后端 voxslice --disp 2260 合主线 a41d63b (独立复验 24/0, 合并后回归 d21/d23 过)</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>D:\card03</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10351,12 +10351,12 @@
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>D25</t>
+          <t>D20e</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>V1 换档合主线 90b1d79: 358/286/210 档 (阈值 11.6/14.6 rps, 回差), 各档最高转速桥余量 3.9/3.3/2.7%; 不改 RTL 不重出位流; 顺修 --local-always SIGTERM 挂死; 卡上 voxslice 仍 D20e 版 (V0 dump 逐字节同, 不急换)</t>
+          <t>推流相位锁定合主线 c80f5fb: 583 rpm 滑格 5.2%→0.19%, 900 rpm 22%→0.12% (p95 = 理想间隔); 代价 延迟 120→170-250 ms (--phaselock off 可回老行为)</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
@@ -10369,24 +10369,24 @@
       <c r="A79" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B79" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>部署</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>用户改供电上电后: mDNS 查不到, 串口 COM29/COM30 (CH342) 140 s 无输出、回车无回显; 后台录串口 2 h + 寻板 3 h; 待用户回来断电重上电</t>
+          <t>02 卡上 voxslice 换 D20e 版 (ba243d71, 旧版留 .bak-d20e), 重启后 V0 验收 6/6 PASS (推流 1326 帧/90 s, WiFi -44 dBm 丢 0)</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>D:\card03\cap_COM29.log</t>
+          <t>progress/v0_accept/accept_1016_d20e.log</t>
         </is>
       </c>
     </row>
@@ -10394,24 +10394,24 @@
       <c r="A80" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B80" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B80" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>回归</t>
+          <t>KR7.3/D24</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>d20d P2 / d20c F3 帧间隔 std 判据在机器高负载 (load 4-6, D25 全量 + D26 TD) 时偶发超门槛 (4.6/8.3 ms vs &lt;4), 空闲同代码 0.1 ms; 待空闲复测, 必要时改失败重测一次</t>
+          <t>KR7.3 16 位计数回绕修正合主线 (存档无原始计数, 99.84% 无法重算; 38/57 转动行待核); D24 立方体候选合主线, 用户定开机保持 geo_loop</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d20d_ackrps d20c_fps</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10419,24 +10419,24 @@
       <c r="A81" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B81" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>硬件</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>延迟复测合主线: 相位锁定 auto 保持, lock-lead 150→70 ms; 583 rpm 延迟 p50/p95/p99 133/138/155 ms (锁相关 126/127/196, 滑格 2.1%→0.14%); 900 rpm 122/206/276 ms 滑格 0.37%; 帧间隔 p95 = 理想</t>
+          <t>第二块板: 公司 DLP 拦 TF 卡文件写入 → WSL 做 512 MB 镜像 + host/flash_card_raw.ps1 块级写, 读回 PASS; 等上电按名字找</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d12_latency/RESULTS.md</t>
+          <t>D:\card03</t>
         </is>
       </c>
     </row>
@@ -10451,17 +10451,17 @@
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>D25</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>V1 端到端仿真合主线: 真内容主机→板端→主控 RTL→上行→桥→6×2260 模型, 逐像素 0 错; 反例 3/3; 358 档只跑回绕窗口 (整圈用 N=16), 只 12-bit/假角度</t>
+          <t>V1 换档合主线 90b1d79: 358/286/210 档 (阈值 11.6/14.6 rps, 回差), 各档最高转速桥余量 3.9/3.3/2.7%; 不改 RTL 不重出位流; 顺修 --local-always SIGTERM 挂死; 卡上 voxslice 仍 D20e 版 (V0 dump 逐字节同, 不急换)</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d9_e2e/</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10469,9 +10469,9 @@
       <c r="A83" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B83" s="6" t="inlineStr">
-        <is>
-          <t>硬件</t>
+      <c r="B83" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
@@ -10481,12 +10481,12 @@
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>03 起来了: 控制台 COM30 (CH342-A); 冷上电 u-boot 报 Card did not respond to voltage select -110 停在 =&gt;, mmc rescan + boot 后正常; 登记 dr1m90-03 (10.10.21.10), V0 验收 6/6 PASS (WiFi -45 dBm, 推流 1351 帧/90 s) → D29 查根因</t>
+          <t>用户改供电上电后: mDNS 查不到, 串口 COM29/COM30 (CH342) 140 s 无输出、回车无回显; 后台录串口 2 h + 寻板 3 h; 待用户回来断电重上电</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>D:\card03\boot03.log</t>
+          <t>D:\card03\cap_COM29.log</t>
         </is>
       </c>
     </row>
@@ -10494,24 +10494,24 @@
       <c r="A84" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B84" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B84" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>D26</t>
+          <t>回归</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>V2 位流按主线重出合主线 c8e8294: 0 违例但余量 0.000 ns (旧 +0.001), 资源略降; D26 agent 遗留的卡死构建进程 (嵌套 flock) 占锁 2.5 h, 已按 PID 清掉</t>
+          <t>d20d P2 / d20c F3 帧间隔 std 判据在机器高负载 (load 4-6, D25 全量 + D26 TD) 时偶发超门槛 (4.6/8.3 ms vs &lt;4), 空闲同代码 0.1 ms; 待空闲复测, 必要时改失败重测一次</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 td_pov/pure_ul/results/p2_ul1200_b12_v3</t>
+          <t>dr1v90 d20d_ackrps d20c_fps</t>
         </is>
       </c>
     </row>
@@ -10519,24 +10519,24 @@
       <c r="A85" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B85" s="6" t="inlineStr">
-        <is>
-          <t>开工</t>
+      <c r="B85" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>周末</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>用户: SoC↔桥通信全功能开工, 软件能做的都做, 周一看结果。开 D27 (SoC↔桥全功能, Opus) / D28 (V1 回板一键脚本) / D29 (冷启动认卡); 02 跑 24 h 产品配置长跑 (PLV=0 max-fps 20 margin 1.0, 主线 8eced5a)</t>
+          <t>延迟复测合主线: 相位锁定 auto 保持, lock-lead 150→70 ms; 583 rpm 延迟 p50/p95/p99 133/138/155 ms (锁相关 126/127/196, 滑格 2.1%→0.14%); 900 rpm 122/206/276 ms 滑格 0.37%; 帧间隔 p95 = 理想</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 soak8h/runs/1016_wkend_24h</t>
+          <t>dr1v90 d12_latency/RESULTS.md</t>
         </is>
       </c>
     </row>
@@ -10544,24 +10544,24 @@
       <c r="A86" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B86" s="6" t="inlineStr">
-        <is>
-          <t>方案</t>
+      <c r="B86" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>D29</t>
+          <t>D9</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>03 冷启动认卡: 热重启 13/13 无法复现, 最可能 u-boot sdhci 首次 mmc_init 间歇失败且 an_bootcmd 无重试; 方案 A 只改卡上 uboot.env 的 bootcmd (mmc rescan 重试 15 次, 其余 49 变量逐字节同, md5 dae13f64), u-boot 提示符手敲已验证; 等用户批准写卡 + 冷上电 20 次验收 (判据 20/20); 发现 03 未装 S00sdoff 钩子</t>
+          <t>V1 端到端仿真合主线: 真内容主机→板端→主控 RTL→上行→桥→6×2260 模型, 逐像素 0 错; 反例 3/3; 358 档只跑回绕窗口 (整圈用 N=16), 只 12-bit/假角度</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d29_sdboot/PLAN.md</t>
+          <t>dr1v90 d9_e2e/</t>
         </is>
       </c>
     </row>
@@ -10569,24 +10569,24 @@
       <c r="A87" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B87" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>硬件</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>D28</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>V1 回板一键脚本合主线: bringup.sh S0 前置 → S9 恢复, 每步 CHECK + 失败原因/下一步; 演练 (假寄存器/qemu) 74 PASS, 12 种故障注入全命中; 待真板核: 位流加载/真线速误码/真画面/桥 UART 字符串</t>
+          <t>03 起来了: 控制台 COM30 (CH342-A); 冷上电 u-boot 报 Card did not respond to voltage select -110 停在 =&gt;, mmc rescan + boot 后正常; 登记 dr1m90-03 (10.10.21.10), V0 验收 6/6 PASS (WiFi -45 dBm, 推流 1351 帧/90 s) → D29 查根因</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v1_bringup/</t>
+          <t>D:\card03\boot03.log</t>
         </is>
       </c>
     </row>
@@ -10594,24 +10594,24 @@
       <c r="A88" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B88" s="6" t="inlineStr">
-        <is>
-          <t>修复</t>
+      <c r="B88" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>D30</t>
+          <t>D26</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>回归计时判据 (d20d P2 / d20c F3) 抗机器忙合主线: 稳健 std + 失败重测; load 17-31 下 5/5 PASS, 反例全检出</t>
+          <t>V2 位流按主线重出合主线 c8e8294: 0 违例但余量 0.000 ns (旧 +0.001), 资源略降; D26 agent 遗留的卡死构建进程 (嵌套 flock) 占锁 2.5 h, 已按 PID 清掉</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d20c_fps/test_d30_judge.sh</t>
+          <t>dr1v90 td_pov/pure_ul/results/p2_ul1200_b12_v3</t>
         </is>
       </c>
     </row>
@@ -10621,22 +10621,22 @@
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>进展</t>
+          <t>开工</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>V2-3</t>
+          <t>周末</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>2 期 192×216 映射离线完成合主线 691a772 (复验 15/15): p2_192x216 profile, 605 档 == 生产表, v2_ref.py/disp_p2.c 与 2 期全链 tb 逐组对拍; 发现 2 期上行 (105.33 µs/片) 比 2260 更紧, 605/512 两档只到 1110 rpm → 建议 605/513/461; 主控缺列序→字槽序格式器 (方案已证); 9 项待硬件确认 (H1-H9); 待用户定档表</t>
+          <t>用户: SoC↔桥通信全功能开工, 软件能做的都做, 周一看结果。开 D27 (SoC↔桥全功能, Opus) / D28 (V1 回板一键脚本) / D29 (冷启动认卡); 02 跑 24 h 产品配置长跑 (PLV=0 max-fps 20 margin 1.0, 主线 8eced5a)</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v2_map/DESIGN.md</t>
+          <t>dr1v90 soak8h/runs/1016_wkend_24h</t>
         </is>
       </c>
     </row>
@@ -10646,28 +10646,28 @@
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>评估</t>
+          <t>方案</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>D31</t>
+          <t>D29</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>V1 偶数片数漏柱: 面 A 过转轴, 偶数后半圈与前半圈取样重合; 两面漏柱 358/286/210 = 124/458/1524 → 357/285/209 = 0/62/467; 只改档表不动 RTL, 桥余量略宽; 另: D25 阈值下 12 rps 落在 286 档; 待用户定</t>
+          <t>03 冷启动认卡: 热重启 13/13 无法复现, 最可能 u-boot sdhci 首次 mmc_init 间歇失败且 an_bootcmd 无重试; 方案 A 只改卡上 uboot.env 的 bootcmd (mmc rescan 重试 15 次, 其余 49 变量逐字节同, md5 dae13f64), u-boot 提示符手敲已验证; 等用户批准写卡 + 冷上电 20 次验收 (判据 20/20); 发现 03 未装 S00sdoff 钩子</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d31_v1odd/REPORT.md</t>
+          <t>dr1v90 d29_sdboot/PLAN.md</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="17" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
@@ -10676,92 +10676,92 @@
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D28</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
+          <t>V1 回板一键脚本合主线: bringup.sh S0 前置 → S9 恢复, 每步 CHECK + 失败原因/下一步; 演练 (假寄存器/qemu) 74 PASS, 12 种故障注入全命中; 待真板核: 位流加载/真线速误码/真画面/桥 UART 字符串</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/report.md</t>
+          <t>dr1v90 v1_bringup/</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="17" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>测量</t>
+          <t>修复</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>QoS</t>
+          <t>D30</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
+          <t>回归计时判据 (d20d P2 / d20c F3) 抗机器忙合主线: 稳健 std + 失败重测; load 17-31 下 5/5 PASS, 反例全检出</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
         <is>
-          <t>~/qos_runs</t>
+          <t>dr1v90 d20c_fps/test_d30_judge.sh</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="17" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>测量</t>
+          <t>进展</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>D16b</t>
+          <t>V2-3</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
+          <t>2 期 192×216 映射离线完成合主线 691a772 (复验 15/15): p2_192x216 profile, 605 档 == 生产表, v2_ref.py/disp_p2.c 与 2 期全链 tb 逐组对拍; 发现 2 期上行 (105.33 µs/片) 比 2260 更紧, 605/512 两档只到 1110 rpm → 建议 605/513/461; 主控缺列序→字槽序格式器 (方案已证); 9 项待硬件确认 (H1-H9); 待用户定档表</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16b-tile 7936b7e</t>
+          <t>dr1v90 v2_map/DESIGN.md</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B94" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+        <v>46311</v>
+      </c>
+      <c r="B94" s="6" t="inlineStr">
+        <is>
+          <t>评估</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D31</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
+          <t>V1 偶数片数漏柱: 面 A 过转轴, 偶数后半圈与前半圈取样重合; 两面漏柱 358/286/210 = 124/458/1524 → 357/285/209 = 0/62/467; 只改档表不动 RTL, 桥余量略宽; 另: D25 阈值下 12 rps 落在 286 档; 待用户定</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>dr1v90 d31_v1odd/REPORT.md</t>
         </is>
       </c>
     </row>
@@ -10769,24 +10769,24 @@
       <c r="A95" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B95" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B95" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
+          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>progress/soak_v0/report.md</t>
         </is>
       </c>
     </row>
@@ -10796,22 +10796,22 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>分析</t>
+          <t>测量</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>V1/V2</t>
+          <t>QoS</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
+          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>budget/rpm_range_2026-10-15.md</t>
+          <t>~/qos_runs</t>
         </is>
       </c>
     </row>
@@ -10819,24 +10819,24 @@
       <c r="A97" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B97" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B97" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>KR7.3</t>
+          <t>D16b</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
+          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>progress/realspin_v0/</t>
+          <t>dr1v90 task/d16b-tile 7936b7e</t>
         </is>
       </c>
     </row>
@@ -10844,9 +10844,9 @@
       <c r="A98" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B98" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B98" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
@@ -10856,12 +10856,12 @@
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
+          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>progress/realspin_v0/</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -10869,9 +10869,9 @@
       <c r="A99" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B99" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B99" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
@@ -10881,12 +10881,12 @@
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
+          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20-smooth 83a5fd7</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -10894,24 +10894,24 @@
       <c r="A100" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B100" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>分析</t>
         </is>
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>V1/V2</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
+          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
         </is>
       </c>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 e215176</t>
+          <t>budget/rpm_range_2026-10-15.md</t>
         </is>
       </c>
     </row>
@@ -10919,24 +10919,24 @@
       <c r="A101" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B101" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B101" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>KR7.3</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
+          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d19-halfrev 1beafa6</t>
+          <t>progress/realspin_v0/</t>
         </is>
       </c>
     </row>
@@ -10944,24 +10944,24 @@
       <c r="A102" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B102" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B102" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>D20b</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
+          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
         </is>
       </c>
       <c r="E102" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20b-sim 9081f62</t>
+          <t>progress/realspin_v0/</t>
         </is>
       </c>
     </row>
@@ -10971,22 +10971,22 @@
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
+          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/merge-d19-d20 106364e</t>
+          <t>dr1v90 task/d20-smooth 83a5fd7</t>
         </is>
       </c>
     </row>
@@ -11001,17 +11001,17 @@
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>D19/D20</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
+          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
         </is>
       </c>
       <c r="E104" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 e215176</t>
         </is>
       </c>
     </row>
@@ -11026,17 +11026,17 @@
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
+          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband adeba44</t>
+          <t>dr1v90 task/d19-halfrev 1beafa6</t>
         </is>
       </c>
     </row>
@@ -11046,22 +11046,22 @@
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>D20/D22</t>
+          <t>D20b</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
+          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
         </is>
       </c>
       <c r="E106" s="7" t="inlineStr">
         <is>
-          <t>~/realspin/tcp</t>
+          <t>dr1v90 task/d20b-sim 9081f62</t>
         </is>
       </c>
     </row>
@@ -11069,24 +11069,24 @@
       <c r="A107" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B107" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B107" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
+          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>dr1v90 task/merge-d19-d20 106364e</t>
         </is>
       </c>
     </row>
@@ -11094,24 +11094,24 @@
       <c r="A108" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B108" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B108" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D19/D20</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
+          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach ee4a55c</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -11126,17 +11126,17 @@
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
+          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20c-fps 338eaaf</t>
+          <t>dr1v90 task/d21-nband adeba44</t>
         </is>
       </c>
     </row>
@@ -11146,22 +11146,22 @@
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>复验</t>
+          <t>根因</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D20/D22</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
+          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
         </is>
       </c>
       <c r="E110" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d20c.v.log</t>
+          <t>~/realspin/tcp</t>
         </is>
       </c>
     </row>
@@ -11169,24 +11169,24 @@
       <c r="A111" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B111" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B111" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
+          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d8-cosim 85dfe51</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -11194,24 +11194,24 @@
       <c r="A112" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B112" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
+          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
         </is>
       </c>
       <c r="E112" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 task/d22-reach ee4a55c</t>
         </is>
       </c>
     </row>
@@ -11221,22 +11221,22 @@
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>测量</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>D22/D20</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
+          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/netdiag_1015_1814</t>
+          <t>dr1v90 task/d20c-fps 338eaaf</t>
         </is>
       </c>
     </row>
@@ -11244,24 +11244,24 @@
       <c r="A114" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B114" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B114" s="6" t="inlineStr">
+        <is>
+          <t>复验</t>
         </is>
       </c>
       <c r="C114" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
+          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d21.board.log</t>
+          <t>~/rv_d20c.v.log</t>
         </is>
       </c>
     </row>
@@ -11269,24 +11269,24 @@
       <c r="A115" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B115" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B115" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C115" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
+          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach</t>
+          <t>dr1v90 task/d8-cosim 85dfe51</t>
         </is>
       </c>
     </row>
@@ -11294,24 +11294,24 @@
       <c r="A116" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B116" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B116" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
+          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
         </is>
       </c>
       <c r="E116" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -11321,22 +11321,22 @@
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>测量</t>
         </is>
       </c>
       <c r="C117" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D22/D20</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
+          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22.board2.log</t>
+          <t>soak_runs/netdiag_1015_1814</t>
         </is>
       </c>
     </row>
@@ -11344,9 +11344,9 @@
       <c r="A118" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B118" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B118" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C118" s="7" t="inlineStr">
@@ -11356,12 +11356,12 @@
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
+          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
         </is>
       </c>
       <c r="E118" s="7" t="inlineStr">
         <is>
-          <t>~/d21b_forensic.log</t>
+          <t>~/rv_d21.board.log</t>
         </is>
       </c>
     </row>
@@ -11369,9 +11369,9 @@
       <c r="A119" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B119" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B119" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C119" s="7" t="inlineStr">
@@ -11381,12 +11381,12 @@
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
+          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach 0d1da09</t>
+          <t>dr1v90 task/d22-reach</t>
         </is>
       </c>
     </row>
@@ -11394,9 +11394,9 @@
       <c r="A120" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B120" s="6" t="inlineStr">
-        <is>
-          <t>验证</t>
+      <c r="B120" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C120" s="7" t="inlineStr">
@@ -11406,12 +11406,12 @@
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
+          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
         </is>
       </c>
       <c r="E120" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22b.board.log</t>
+          <t>dr1v90 task/d22-reach</t>
         </is>
       </c>
     </row>
@@ -11421,7 +11421,7 @@
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C121" s="7" t="inlineStr">
@@ -11431,12 +11431,12 @@
       </c>
       <c r="D121" s="7" t="inlineStr">
         <is>
-          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
+          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach e438a12</t>
+          <t>~/rv_d22.board2.log</t>
         </is>
       </c>
     </row>
@@ -11456,112 +11456,112 @@
       </c>
       <c r="D122" s="7" t="inlineStr">
         <is>
-          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
+          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
         </is>
       </c>
       <c r="E122" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband 084bba3</t>
+          <t>~/d21b_forensic.log</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B123" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46310</v>
+      </c>
+      <c r="B123" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C123" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
-          <t>上行出口全量复验 45/0, 合主线</t>
+          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 fdb4de6</t>
+          <t>dr1v90 task/d22-reach 0d1da09</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B124" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+        <v>46310</v>
+      </c>
+      <c r="B124" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C124" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
-          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
+          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
         </is>
       </c>
       <c r="E124" s="7" t="inlineStr">
         <is>
-          <t>scratchpad/v_pls4_board.log</t>
+          <t>~/rv_d22b.board.log</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B125" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46310</v>
+      </c>
+      <c r="B125" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C125" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D125" s="7" t="inlineStr">
         <is>
-          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
+          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>dr1v90 task/d22-reach e438a12</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B126" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46310</v>
+      </c>
+      <c r="B126" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
+          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
         </is>
       </c>
       <c r="E126" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>dr1v90 task/d21-nband 084bba3</t>
         </is>
       </c>
     </row>
@@ -11569,24 +11569,24 @@
       <c r="A127" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B127" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B127" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D127" s="7" t="inlineStr">
         <is>
-          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
+          <t>上行出口全量复验 45/0, 合主线</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>project_short_term_delivery_1013</t>
+          <t>dr1v90 fdb4de6</t>
         </is>
       </c>
     </row>
@@ -11594,9 +11594,9 @@
       <c r="A128" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B128" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B128" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C128" s="7" t="inlineStr">
@@ -11606,12 +11606,12 @@
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
+          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
         </is>
       </c>
       <c r="E128" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 debd3cd</t>
+          <t>scratchpad/v_pls4_board.log</t>
         </is>
       </c>
     </row>
@@ -11619,24 +11619,24 @@
       <c r="A129" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B129" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B129" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
+          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>scratchpad v_pls6_board.log</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -11644,24 +11644,24 @@
       <c r="A130" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B130" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B130" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C130" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
+          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
         </is>
       </c>
       <c r="E130" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -11669,24 +11669,24 @@
       <c r="A131" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B131" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B131" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C131" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D131" s="7" t="inlineStr">
         <is>
-          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
+          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16-ddr 539d303</t>
+          <t>project_short_term_delivery_1013</t>
         </is>
       </c>
     </row>
@@ -11694,24 +11694,24 @@
       <c r="A132" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B132" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B132" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
+          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
         </is>
       </c>
       <c r="E132" s="7" t="inlineStr">
         <is>
-          <t>feedback_save_weekly_quota</t>
+          <t>dr1v90 task/pls-2047 debd3cd</t>
         </is>
       </c>
     </row>
@@ -11719,24 +11719,24 @@
       <c r="A133" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B133" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B133" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C133" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D133" s="7" t="inlineStr">
         <is>
-          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
+          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>scratchpad v_pls6_board.log</t>
         </is>
       </c>
     </row>
@@ -11746,7 +11746,7 @@
       </c>
       <c r="B134" s="11" t="inlineStr">
         <is>
-          <t>交付完成</t>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C134" s="7" t="inlineStr">
@@ -11756,12 +11756,12 @@
       </c>
       <c r="D134" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
+          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
         </is>
       </c>
       <c r="E134" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 2364e5c</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -11769,24 +11769,24 @@
       <c r="A135" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B135" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B135" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C135" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D135" s="7" t="inlineStr">
         <is>
-          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
+          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
         <is>
-          <t>用户在场实转</t>
+          <t>dr1v90 task/d16-ddr 539d303</t>
         </is>
       </c>
     </row>
@@ -11801,17 +11801,17 @@
       </c>
       <c r="C136" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
+          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
         </is>
       </c>
       <c r="E136" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>feedback_save_weekly_quota</t>
         </is>
       </c>
     </row>
@@ -11819,24 +11819,24 @@
       <c r="A137" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B137" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B137" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C137" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D137" s="7" t="inlineStr">
         <is>
-          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
+          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
         </is>
       </c>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -11844,24 +11844,24 @@
       <c r="A138" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B138" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B138" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C138" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D138" s="7" t="inlineStr">
         <is>
-          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
+          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
         </is>
       </c>
       <c r="E138" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 2364e5c</t>
         </is>
       </c>
     </row>
@@ -11869,24 +11869,24 @@
       <c r="A139" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B139" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B139" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C139" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D139" s="7" t="inlineStr">
         <is>
-          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
+          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
         </is>
       </c>
       <c r="E139" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 dee9be6</t>
+          <t>用户在场实转</t>
         </is>
       </c>
     </row>
@@ -11894,24 +11894,24 @@
       <c r="A140" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B140" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B140" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C140" s="7" t="inlineStr">
         <is>
-          <t>D15b</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
+          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
         </is>
       </c>
       <c r="E140" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d15b-color-p2</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -11926,17 +11926,17 @@
       </c>
       <c r="C141" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D141" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
+          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
         </is>
       </c>
       <c r="E141" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 3a41eb7</t>
+          <t>dr1v90 task/d18-pl-default d35c6d4</t>
         </is>
       </c>
     </row>
@@ -11944,24 +11944,24 @@
       <c r="A142" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B142" s="6" t="inlineStr">
-        <is>
-          <t>开始</t>
+      <c r="B142" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C142" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D142" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
+          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
         </is>
       </c>
       <c r="E142" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 26e69ec soak8h</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -11969,24 +11969,24 @@
       <c r="A143" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B143" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B143" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C143" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D143" s="7" t="inlineStr">
         <is>
-          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
+          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 dee9be6</t>
         </is>
       </c>
     </row>
@@ -11994,30 +11994,30 @@
       <c r="A144" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B144" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B144" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C144" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D15b</t>
         </is>
       </c>
       <c r="D144" s="7" t="inlineStr">
         <is>
-          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
+          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
         </is>
       </c>
       <c r="E144" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 5cbe79f</t>
+          <t>dr1v90 task/d15b-color-p2</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="17" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B145" s="11" t="inlineStr">
         <is>
@@ -12026,73 +12026,73 @@
       </c>
       <c r="C145" s="7" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D145" s="7" t="inlineStr">
         <is>
-          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
+          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 b0f6b5d</t>
+          <t>dr1v90 3a41eb7</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B146" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B146" s="6" t="inlineStr">
+        <is>
+          <t>开始</t>
         </is>
       </c>
       <c r="C146" s="7" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D146" s="7" t="inlineStr">
         <is>
-          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
+          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
         </is>
       </c>
       <c r="E146" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 71d006f / 473abcf</t>
+          <t>dr1v90 26e69ec soak8h</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B147" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B147" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C147" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D147" s="7" t="inlineStr">
         <is>
-          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
+          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 596b191</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="17" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B148" s="15" t="inlineStr">
         <is>
@@ -12101,17 +12101,17 @@
       </c>
       <c r="C148" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D148" s="7" t="inlineStr">
         <is>
-          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
+          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
         </is>
       </c>
       <c r="E148" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 60c619a / 596b191</t>
+          <t>dr1v90 5cbe79f</t>
         </is>
       </c>
     </row>
@@ -12121,22 +12121,22 @@
       </c>
       <c r="B149" s="11" t="inlineStr">
         <is>
-          <t>复验通过</t>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C149" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="D149" s="7" t="inlineStr">
         <is>
-          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
+          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 9bf16ad</t>
+          <t>dr1v90 b0f6b5d</t>
         </is>
       </c>
     </row>
@@ -12144,24 +12144,24 @@
       <c r="A150" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B150" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B150" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C150" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="D150" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
+          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
         </is>
       </c>
       <c r="E150" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 71d006f / 473abcf</t>
         </is>
       </c>
     </row>
@@ -12171,22 +12171,22 @@
       </c>
       <c r="B151" s="11" t="inlineStr">
         <is>
-          <t>复验通过</t>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C151" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D151" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
+          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 6a373d3</t>
+          <t>dr1v90 596b191</t>
         </is>
       </c>
     </row>
@@ -12194,24 +12194,24 @@
       <c r="A152" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B152" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B152" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C152" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D152" s="7" t="inlineStr">
         <is>
-          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
+          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
         </is>
       </c>
       <c r="E152" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 cdf49c6</t>
+          <t>dr1v90 60c619a / 596b191</t>
         </is>
       </c>
     </row>
@@ -12219,24 +12219,24 @@
       <c r="A153" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B153" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B153" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C153" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D153" s="7" t="inlineStr">
         <is>
-          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
+          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
         </is>
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 9bf16ad</t>
         </is>
       </c>
     </row>
@@ -12244,19 +12244,19 @@
       <c r="A154" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B154" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B154" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C154" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D154" s="7" t="inlineStr">
         <is>
-          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
+          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
         </is>
       </c>
       <c r="E154" s="7" t="inlineStr">
@@ -12276,17 +12276,17 @@
       </c>
       <c r="C155" s="7" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D155" s="7" t="inlineStr">
         <is>
-          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
+          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 44ed2cd</t>
+          <t>dr1v90 6a373d3</t>
         </is>
       </c>
     </row>
@@ -12294,24 +12294,24 @@
       <c r="A156" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B156" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B156" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C156" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D156" s="7" t="inlineStr">
         <is>
-          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
+          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
         </is>
       </c>
       <c r="E156" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 cdf49c6</t>
         </is>
       </c>
     </row>
@@ -12319,24 +12319,24 @@
       <c r="A157" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B157" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B157" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C157" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D157" s="7" t="inlineStr">
         <is>
-          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
+          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ffbfeeb</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12344,19 +12344,19 @@
       <c r="A158" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B158" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B158" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C158" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D158" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
+          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
         </is>
       </c>
       <c r="E158" s="7" t="inlineStr">
@@ -12369,24 +12369,24 @@
       <c r="A159" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B159" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B159" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C159" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="D159" s="7" t="inlineStr">
         <is>
-          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
+          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 44ed2cd</t>
         </is>
       </c>
     </row>
@@ -12394,24 +12394,24 @@
       <c r="A160" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B160" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B160" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C160" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D160" s="7" t="inlineStr">
         <is>
-          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
+          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
         </is>
       </c>
       <c r="E160" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 764f81d</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12419,24 +12419,24 @@
       <c r="A161" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B161" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B161" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C161" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D161" s="7" t="inlineStr">
         <is>
-          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
+          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 ffbfeeb</t>
         </is>
       </c>
     </row>
@@ -12444,24 +12444,24 @@
       <c r="A162" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B162" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B162" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C162" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D162" s="7" t="inlineStr">
         <is>
-          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
+          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
         </is>
       </c>
       <c r="E162" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d13-boot fdbb217</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12469,19 +12469,19 @@
       <c r="A163" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B163" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B163" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C163" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D163" s="7" t="inlineStr">
         <is>
-          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
+          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
         </is>
       </c>
       <c r="E163" s="7" t="inlineStr">
@@ -12494,24 +12494,24 @@
       <c r="A164" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B164" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B164" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C164" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D164" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
+          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
         </is>
       </c>
       <c r="E164" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 1995be8</t>
+          <t>dr1v90 764f81d</t>
         </is>
       </c>
     </row>
@@ -12519,19 +12519,19 @@
       <c r="A165" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B165" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B165" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C165" s="7" t="inlineStr">
         <is>
-          <t>D3;D4;D5</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D165" s="7" t="inlineStr">
         <is>
-          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
+          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
         </is>
       </c>
       <c r="E165" s="7" t="inlineStr">
@@ -12544,20 +12544,24 @@
       <c r="A166" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B166" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C166" s="7" t="inlineStr"/>
+      <c r="B166" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
+        </is>
+      </c>
+      <c r="C166" s="7" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
       <c r="D166" s="7" t="inlineStr">
         <is>
-          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
+          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
         </is>
       </c>
       <c r="E166" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>dr1v90 task/d13-boot fdbb217</t>
         </is>
       </c>
     </row>
@@ -12565,20 +12569,24 @@
       <c r="A167" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B167" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
-        </is>
-      </c>
-      <c r="C167" s="7" t="inlineStr"/>
+      <c r="B167" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C167" s="7" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
       <c r="D167" s="7" t="inlineStr">
         <is>
-          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
+          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
         </is>
       </c>
       <c r="E167" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12586,20 +12594,24 @@
       <c r="A168" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B168" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C168" s="7" t="inlineStr"/>
+      <c r="B168" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
+        </is>
+      </c>
+      <c r="C168" s="7" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
       <c r="D168" s="7" t="inlineStr">
         <is>
-          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
+          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
         </is>
       </c>
       <c r="E168" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_arch_common_front_display_backend.md</t>
+          <t>dr1v90 1995be8</t>
         </is>
       </c>
     </row>
@@ -12614,12 +12626,12 @@
       </c>
       <c r="C169" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D3;D4;D5</t>
         </is>
       </c>
       <c r="D169" s="7" t="inlineStr">
         <is>
-          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
+          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
         </is>
       </c>
       <c r="E169" s="7" t="inlineStr">
@@ -12637,19 +12649,15 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C170" s="7" t="inlineStr">
-        <is>
-          <t>D11</t>
-        </is>
-      </c>
+      <c r="C170" s="7" t="inlineStr"/>
       <c r="D170" s="7" t="inlineStr">
         <is>
-          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
+          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
         </is>
       </c>
       <c r="E170" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -12657,24 +12665,20 @@
       <c r="A171" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B171" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C171" s="7" t="inlineStr">
-        <is>
-          <t>D12;D13;D14</t>
-        </is>
-      </c>
+      <c r="B171" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
+        </is>
+      </c>
+      <c r="C171" s="7" t="inlineStr"/>
       <c r="D171" s="7" t="inlineStr">
         <is>
-          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
+          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
         </is>
       </c>
       <c r="E171" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -12687,19 +12691,15 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C172" s="7" t="inlineStr">
-        <is>
-          <t>D13</t>
-        </is>
-      </c>
+      <c r="C172" s="7" t="inlineStr"/>
       <c r="D172" s="7" t="inlineStr">
         <is>
-          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
         </is>
       </c>
       <c r="E172" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_arch_common_front_display_backend.md</t>
         </is>
       </c>
     </row>
@@ -12714,12 +12714,12 @@
       </c>
       <c r="C173" s="7" t="inlineStr">
         <is>
-          <t>D15;D16</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D173" s="7" t="inlineStr">
         <is>
-          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
         </is>
       </c>
       <c r="E173" s="7" t="inlineStr">
@@ -12739,17 +12739,17 @@
       </c>
       <c r="C174" s="7" t="inlineStr">
         <is>
-          <t>KR5.2</t>
+          <t>D11</t>
         </is>
       </c>
       <c r="D174" s="7" t="inlineStr">
         <is>
-          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
         </is>
       </c>
       <c r="E174" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 49031f6</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12757,19 +12757,19 @@
       <c r="A175" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B175" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B175" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C175" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D12;D13;D14</t>
         </is>
       </c>
       <c r="D175" s="7" t="inlineStr">
         <is>
-          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
         </is>
       </c>
       <c r="E175" s="7" t="inlineStr">
@@ -12782,18 +12782,118 @@
       <c r="A176" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B176" s="19" t="inlineStr">
+      <c r="B176" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C176" s="7" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="D176" s="7" t="inlineStr">
+        <is>
+          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+        </is>
+      </c>
+      <c r="E176" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B177" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C177" s="7" t="inlineStr">
+        <is>
+          <t>D15;D16</t>
+        </is>
+      </c>
+      <c r="D177" s="7" t="inlineStr">
+        <is>
+          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+        </is>
+      </c>
+      <c r="E177" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B178" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C178" s="7" t="inlineStr">
+        <is>
+          <t>KR5.2</t>
+        </is>
+      </c>
+      <c r="D178" s="7" t="inlineStr">
+        <is>
+          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+        </is>
+      </c>
+      <c r="E178" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 49031f6</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B179" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C179" s="7" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="D179" s="7" t="inlineStr">
+        <is>
+          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+        </is>
+      </c>
+      <c r="E179" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B180" s="19" t="inlineStr">
         <is>
           <t>里程碑</t>
         </is>
       </c>
-      <c r="C176" s="7" t="inlineStr"/>
-      <c r="D176" s="7" t="inlineStr">
+      <c r="C180" s="7" t="inlineStr"/>
+      <c r="D180" s="7" t="inlineStr">
         <is>
           <t>显性目的进度看板第一版建立：10 个显性目的 + KR 趋势 + 燃起图 + 里程碑趋势</t>
         </is>
       </c>
-      <c r="E176" s="7" t="inlineStr">
+      <c r="E180" s="7" t="inlineStr">
         <is>
           <t>claude_memory/project_progress_dashboard.md</t>
         </is>

</xml_diff>